<commit_message>
so many adds to Cij plotting
</commit_message>
<xml_diff>
--- a/Vanadium_Cij_finite_strain_all_equations_GlobalMin - Copy.xlsx
+++ b/Vanadium_Cij_finite_strain_all_equations_GlobalMin - Copy.xlsx
@@ -8,211 +8,212 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bgulick\Downloads\vCIJ_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8C82B5-3C42-4F86-99C6-27A640B5F169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5922B096-8A0F-4CF2-BF6C-7F21E16C8C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F35EC34-C410-40C3-9DB6-F447C7BA1DCF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F35EC34-C410-40C3-9DB6-F447C7BA1DCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="5" r:id="rId1"/>
     <sheet name="Cook updated" sheetId="6" r:id="rId2"/>
     <sheet name="data" sheetId="9" r:id="rId3"/>
     <sheet name="FS No Vs 111" sheetId="1" r:id="rId4"/>
-    <sheet name="FS No Vp 111" sheetId="2" r:id="rId5"/>
-    <sheet name="FS No Vs 100" sheetId="3" r:id="rId6"/>
-    <sheet name="FS No Vp 100" sheetId="4" r:id="rId7"/>
-    <sheet name="TRUE GLOBAL" sheetId="7" r:id="rId8"/>
-    <sheet name="TRUE GLOBAL (2)" sheetId="8" r:id="rId9"/>
+    <sheet name="Katahara extrap" sheetId="10" r:id="rId5"/>
+    <sheet name="FS No Vp 111" sheetId="2" r:id="rId6"/>
+    <sheet name="FS No Vs 100" sheetId="3" r:id="rId7"/>
+    <sheet name="FS No Vp 100" sheetId="4" r:id="rId8"/>
+    <sheet name="TRUE GLOBAL" sheetId="7" r:id="rId9"/>
+    <sheet name="TRUE GLOBAL (2)" sheetId="8" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="1" hidden="1">'Cook updated'!$AN$3:$AN$16,'Cook updated'!$AP$25:$AP$27,'Cook updated'!$AR$25:$AR$27</definedName>
-    <definedName name="solver_adj" localSheetId="6" hidden="1">'FS No Vp 100'!$AS$26:$AS$28,'FS No Vp 100'!$AS$29:$AS$31</definedName>
-    <definedName name="solver_adj" localSheetId="4" hidden="1">'FS No Vp 111'!$AQ$28:$AQ$30,'FS No Vp 111'!$AQ$31:$AQ$33</definedName>
-    <definedName name="solver_adj" localSheetId="5" hidden="1">'FS No Vs 100'!$AQ$26:$AQ$28,'FS No Vs 100'!$AQ$29:$AQ$31</definedName>
+    <definedName name="solver_adj" localSheetId="7" hidden="1">'FS No Vp 100'!$AS$26:$AS$28,'FS No Vp 100'!$AS$29:$AS$31</definedName>
+    <definedName name="solver_adj" localSheetId="5" hidden="1">'FS No Vp 111'!$AQ$28:$AQ$30,'FS No Vp 111'!$AQ$31:$AQ$33</definedName>
+    <definedName name="solver_adj" localSheetId="6" hidden="1">'FS No Vs 100'!$AQ$26:$AQ$28,'FS No Vs 100'!$AQ$29:$AQ$31</definedName>
     <definedName name="solver_adj" localSheetId="3" hidden="1">'FS No Vs 111'!$AP$26:$AP$28,'FS No Vs 111'!$AR$26:$AR$28</definedName>
-    <definedName name="solver_adj" localSheetId="7" hidden="1">'TRUE GLOBAL'!$M$12:$M$17,'TRUE GLOBAL'!$M$31:$M$52</definedName>
-    <definedName name="solver_adj" localSheetId="8" hidden="1">'TRUE GLOBAL (2)'!$M$12:$M$17,'TRUE GLOBAL (2)'!$M$31:$M$52</definedName>
+    <definedName name="solver_adj" localSheetId="8" hidden="1">'TRUE GLOBAL'!$M$12:$M$17,'TRUE GLOBAL'!$M$31:$M$52</definedName>
+    <definedName name="solver_adj" localSheetId="9" hidden="1">'TRUE GLOBAL (2)'!$M$12:$M$17,'TRUE GLOBAL (2)'!$M$31:$M$52</definedName>
     <definedName name="solver_cvg" localSheetId="1" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="4" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="3" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="8" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="9" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_drv" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_drv" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="9" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="9" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="9" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="9" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="1" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="4" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="3" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="8" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="9" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="1" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="4" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="3" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="8" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="9" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="4" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="9" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="9" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_num" localSheetId="7" hidden="1">0</definedName>
+    <definedName name="solver_num" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_num" localSheetId="6" hidden="1">0</definedName>
-    <definedName name="solver_num" localSheetId="4" hidden="1">0</definedName>
-    <definedName name="solver_num" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_num" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_num" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_num" localSheetId="8" hidden="1">0</definedName>
+    <definedName name="solver_num" localSheetId="9" hidden="1">0</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="9" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">'Cook updated'!$AT$32</definedName>
-    <definedName name="solver_opt" localSheetId="6" hidden="1">'FS No Vp 100'!$AS$32</definedName>
-    <definedName name="solver_opt" localSheetId="4" hidden="1">'FS No Vp 111'!$AQ$34</definedName>
-    <definedName name="solver_opt" localSheetId="5" hidden="1">'FS No Vs 100'!$AQ$32</definedName>
+    <definedName name="solver_opt" localSheetId="7" hidden="1">'FS No Vp 100'!$AS$32</definedName>
+    <definedName name="solver_opt" localSheetId="5" hidden="1">'FS No Vp 111'!$AQ$34</definedName>
+    <definedName name="solver_opt" localSheetId="6" hidden="1">'FS No Vs 100'!$AQ$32</definedName>
     <definedName name="solver_opt" localSheetId="3" hidden="1">'FS No Vs 111'!$AV$30</definedName>
-    <definedName name="solver_opt" localSheetId="7" hidden="1">'TRUE GLOBAL'!$B$24</definedName>
-    <definedName name="solver_opt" localSheetId="8" hidden="1">'TRUE GLOBAL (2)'!$B$24</definedName>
+    <definedName name="solver_opt" localSheetId="8" hidden="1">'TRUE GLOBAL'!$B$24</definedName>
+    <definedName name="solver_opt" localSheetId="9" hidden="1">'TRUE GLOBAL (2)'!$B$24</definedName>
     <definedName name="solver_pre" localSheetId="1" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
-    <definedName name="solver_pre" localSheetId="4" hidden="1">0.000001</definedName>
-    <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0.000001</definedName>
-    <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="8" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="9" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_rbv" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_rbv" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rbv" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_rbv" localSheetId="4" hidden="1">2</definedName>
-    <definedName name="solver_rbv" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rbv" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_rbv" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_rbv" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_rbv" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="4" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="4" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="8" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="9" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_scl" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_scl" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_scl" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="4" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_ssz" localSheetId="1" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
-    <definedName name="solver_ssz" localSheetId="4" hidden="1">100</definedName>
-    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="3" hidden="1">100</definedName>
-    <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="8" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="9" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="9" hidden="1">2147483647</definedName>
     <definedName name="solver_tol" localSheetId="1" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="4" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="3" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="8" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="9" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="4" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="8" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="9" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="7" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="7" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="8" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="9" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -238,7 +239,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="248">
   <si>
     <t>V100 Pressure</t>
   </si>
@@ -890,6 +891,99 @@
   <si>
     <t>Oil P 111</t>
   </si>
+  <si>
+    <t>KATAHARA 1979  (V, 298 K)</t>
+  </si>
+  <si>
+    <t>C11_0 (GPa)</t>
+  </si>
+  <si>
+    <t>C12_0 (GPa)</t>
+  </si>
+  <si>
+    <t>C44_0 (GPa)</t>
+  </si>
+  <si>
+    <t>dC11/dP</t>
+  </si>
+  <si>
+    <t>dC12/dP</t>
+  </si>
+  <si>
+    <t>dC44/dP</t>
+  </si>
+  <si>
+    <t>C'_0</t>
+  </si>
+  <si>
+    <t>dC'/dP</t>
+  </si>
+  <si>
+    <t>K0</t>
+  </si>
+  <si>
+    <t>K0'</t>
+  </si>
+  <si>
+    <t>P meas (GPa)</t>
+  </si>
+  <si>
+    <t>V0/V</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>P BM3 kat</t>
+  </si>
+  <si>
+    <t>C11 lin</t>
+  </si>
+  <si>
+    <t>C12 lin</t>
+  </si>
+  <si>
+    <t>C44 lin</t>
+  </si>
+  <si>
+    <t>C' lin</t>
+  </si>
+  <si>
+    <t>K lin</t>
+  </si>
+  <si>
+    <t>C11 FS</t>
+  </si>
+  <si>
+    <t>C12 FS</t>
+  </si>
+  <si>
+    <t>C44 FS</t>
+  </si>
+  <si>
+    <t>C' FS</t>
+  </si>
+  <si>
+    <t>K FS</t>
+  </si>
+  <si>
+    <t>C11 mine</t>
+  </si>
+  <si>
+    <t>C12 mine</t>
+  </si>
+  <si>
+    <t>C44 mine</t>
+  </si>
+  <si>
+    <t>dC11 FS-mine</t>
+  </si>
+  <si>
+    <t>dC12 FS-mine</t>
+  </si>
+  <si>
+    <t>dC44 FS-mine</t>
+  </si>
 </sst>
 </file>
 
@@ -903,7 +997,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1006,6 +1100,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -1105,7 +1207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1248,6 +1350,7 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5182,6 +5285,925 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12A38178-9331-4F70-84AF-90930ECA28C5}">
+  <dimension ref="A1:S52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="15" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H3" t="s">
+        <v>164</v>
+      </c>
+      <c r="I3" t="s">
+        <v>165</v>
+      </c>
+      <c r="J3" t="s">
+        <v>166</v>
+      </c>
+      <c r="K3" t="s">
+        <v>167</v>
+      </c>
+      <c r="L3" t="s">
+        <v>168</v>
+      </c>
+      <c r="M3" t="s">
+        <v>169</v>
+      </c>
+      <c r="N3" t="s">
+        <v>170</v>
+      </c>
+      <c r="O3" t="s">
+        <v>171</v>
+      </c>
+      <c r="P3" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>173</v>
+      </c>
+      <c r="S3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="103">
+        <f>'FS No Vs 111'!BG25</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="C4" s="103">
+        <f>'FS No Vp 111'!BC25</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="D4" s="103">
+        <f>'FS No Vs 100'!BF25</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="E4" s="103">
+        <f>'FS No Vp 100'!BH25</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="F4" s="103">
+        <f>'FS No Vs 111'!AP26</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="G4" s="103">
+        <f>'FS No Vp 111'!AQ28</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="H4" s="103">
+        <f>'FS No Vs 100'!AQ26</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="I4" s="103">
+        <f>'FS No Vp 100'!AS26</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:K9" si="0">AVERAGE(B4:E4)</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ref="L4:L9" si="1">AVERAGE(F4:I4)</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="M4">
+        <f t="shared" ref="M4:M9" si="2">AVERAGE(B4:I4)</f>
+        <v>239.73960242643554</v>
+      </c>
+      <c r="N4">
+        <f t="shared" ref="N4:N9" si="3">J4*IF($D$11=1,DEVSQ(B4:E4)/K4^2,DEVSQ(B4:E4))</f>
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <f t="shared" ref="O4:O9" si="4">J4*IF($D$11=1,DEVSQ(F4:I4)/L4^2,DEVSQ(F4:I4))</f>
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <f t="shared" ref="P4:P9" si="5">J4*IF($D$11=1,(K4-L4)^2/M4^2,(K4-L4)^2)</f>
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" ref="Q4:Q9" si="6">J4*IF($D$11=1,DEVSQ(B4:I4)/M4^2,DEVSQ(B4:I4))</f>
+        <v>6.4623485355705287E-27</v>
+      </c>
+      <c r="S4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="103">
+        <f>'FS No Vs 111'!BG26</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="C5" s="103">
+        <f>'FS No Vp 111'!BC26</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="D5" s="103">
+        <f>'FS No Vs 100'!BF26</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="E5" s="103">
+        <f>'FS No Vp 100'!BH26</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="F5" s="103">
+        <f>'FS No Vs 111'!AP27</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="G5" s="103">
+        <f>'FS No Vp 111'!AQ29</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="H5" s="103">
+        <f>'FS No Vs 100'!AQ27</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="I5" s="103">
+        <f>'FS No Vp 100'!AS27</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="0"/>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="1"/>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="2"/>
+        <v>121.94076995584668</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="6"/>
+        <v>1.6155871338926322E-27</v>
+      </c>
+      <c r="S5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="103">
+        <f>'FS No Vs 111'!BG27</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="C6" s="103">
+        <f>'FS No Vp 111'!BC27</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="D6" s="103">
+        <f>'FS No Vs 100'!BF27</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="E6" s="103">
+        <f>'FS No Vp 100'!BH27</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="F6" s="103">
+        <f>'FS No Vs 111'!AP28</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="G6" s="103">
+        <f>'FS No Vp 111'!AQ30</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="H6" s="103">
+        <f>'FS No Vs 100'!AQ28</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="I6" s="103">
+        <f>'FS No Vp 100'!AS28</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="0"/>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="1"/>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="2"/>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="S6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="103">
+        <f>'FS No Vs 111'!BG28</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="C7" s="103">
+        <f>'FS No Vp 111'!BC28</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="D7" s="103">
+        <f>'FS No Vs 100'!BF28</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="E7" s="103">
+        <f>'FS No Vp 100'!BH28</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="F7" s="103">
+        <f>'FS No Vs 111'!AR26</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="G7" s="103">
+        <f>'FS No Vp 111'!AQ31</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="H7" s="103">
+        <f>'FS No Vs 100'!AQ29</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="I7" s="103">
+        <f>'FS No Vp 100'!AS29</f>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="0"/>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="1"/>
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="2"/>
+        <v>5.4435182877526822</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="S7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="103">
+        <f>'FS No Vs 111'!BG29</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="C8" s="103">
+        <f>'FS No Vp 111'!BC29</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="D8" s="103">
+        <f>'FS No Vs 100'!BF29</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="E8" s="103">
+        <f>'FS No Vp 100'!BH29</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="F8" s="103">
+        <f>'FS No Vs 111'!AR27</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="G8" s="103">
+        <f>'FS No Vp 111'!AQ32</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="H8" s="103">
+        <f>'FS No Vs 100'!AQ30</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="I8" s="103">
+        <f>'FS No Vp 100'!AS30</f>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="0"/>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="1"/>
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="2"/>
+        <v>3.0672134474127288</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="S8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="103">
+        <f>'FS No Vs 111'!BG30</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="C9" s="103">
+        <f>'FS No Vp 111'!BC30</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="D9" s="103">
+        <f>'FS No Vs 100'!BF30</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="E9" s="103">
+        <f>'FS No Vp 100'!BH30</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="F9" s="103">
+        <f>'FS No Vs 111'!AR28</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="G9" s="103">
+        <f>'FS No Vp 111'!AQ33</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="H9" s="103">
+        <f>'FS No Vs 100'!AQ31</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="I9" s="103">
+        <f>'FS No Vp 100'!AS31</f>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="0"/>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="1"/>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="2"/>
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="S9" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>181</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="L11" t="s">
+        <v>203</v>
+      </c>
+      <c r="M11" t="s">
+        <v>205</v>
+      </c>
+      <c r="S11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="K12" t="s">
+        <v>62</v>
+      </c>
+      <c r="L12">
+        <v>239.73960242643551</v>
+      </c>
+      <c r="M12">
+        <v>239.510382116199</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>183</v>
+      </c>
+      <c r="E13">
+        <f>SUM(N4:N9)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" t="s">
+        <v>66</v>
+      </c>
+      <c r="L13">
+        <v>121.94076995584666</v>
+      </c>
+      <c r="M13">
+        <v>121.79137881717247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>184</v>
+      </c>
+      <c r="E14">
+        <f>SUM(O4:O9)</f>
+        <v>0</v>
+      </c>
+      <c r="K14" t="s">
+        <v>71</v>
+      </c>
+      <c r="L14">
+        <v>46.232580877717901</v>
+      </c>
+      <c r="M14">
+        <v>46.243127016089062</v>
+      </c>
+      <c r="S14" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>186</v>
+      </c>
+      <c r="E15">
+        <f>SUM(P4:P9)</f>
+        <v>0</v>
+      </c>
+      <c r="K15" t="s">
+        <v>63</v>
+      </c>
+      <c r="L15">
+        <v>5.4435182877526831</v>
+      </c>
+      <c r="M15">
+        <v>5.5155923611825912</v>
+      </c>
+      <c r="S15" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>188</v>
+      </c>
+      <c r="E16">
+        <f>SUM(Q4:Q9)</f>
+        <v>8.0779356694631609E-27</v>
+      </c>
+      <c r="K16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16">
+        <v>3.0672134474127284</v>
+      </c>
+      <c r="M16">
+        <v>3.112817975691188</v>
+      </c>
+      <c r="S16" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K17" t="s">
+        <v>72</v>
+      </c>
+      <c r="L17">
+        <v>0.28956719904890593</v>
+      </c>
+      <c r="M17">
+        <v>0.28796770498141772</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>191</v>
+      </c>
+      <c r="B19" t="s">
+        <v>192</v>
+      </c>
+      <c r="C19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20">
+        <f>'FS No Vs 111'!BG31</f>
+        <v>7.2180533228467745</v>
+      </c>
+      <c r="C20">
+        <f>'FS No Vs 111'!AV30</f>
+        <v>55.456507868353405</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>195</v>
+      </c>
+      <c r="B21">
+        <f>'FS No Vp 111'!BC31</f>
+        <v>52.196130402976017</v>
+      </c>
+      <c r="C21">
+        <f>'FS No Vp 111'!AQ34</f>
+        <v>983.36124073377607</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22">
+        <f>'FS No Vs 100'!BF31</f>
+        <v>15.798705890900674</v>
+      </c>
+      <c r="C22">
+        <f>'FS No Vs 100'!AQ32</f>
+        <v>18.827546785413528</v>
+      </c>
+      <c r="L22" t="s">
+        <v>202</v>
+      </c>
+      <c r="M22" t="s">
+        <v>201</v>
+      </c>
+      <c r="N22" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B23">
+        <f>'FS No Vp 100'!BH31</f>
+        <v>11.333238543153788</v>
+      </c>
+      <c r="C23">
+        <f>'FS No Vp 100'!AS32</f>
+        <v>74.737893177232252</v>
+      </c>
+      <c r="K23" t="s">
+        <v>62</v>
+      </c>
+      <c r="L23">
+        <v>239.89360432346049</v>
+      </c>
+      <c r="M23">
+        <v>239.510382116199</v>
+      </c>
+      <c r="N23">
+        <v>239.73960250702001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>198</v>
+      </c>
+      <c r="B24">
+        <f>SUM(B20:B23)</f>
+        <v>86.546128159877256</v>
+      </c>
+      <c r="C24">
+        <f>SUM(C20:C23)</f>
+        <v>1132.3831885647753</v>
+      </c>
+      <c r="K24" t="s">
+        <v>66</v>
+      </c>
+      <c r="L24">
+        <v>122.04281469011407</v>
+      </c>
+      <c r="M24">
+        <v>121.79137881717247</v>
+      </c>
+      <c r="N24">
+        <v>121.94076993310495</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>199</v>
+      </c>
+      <c r="B25">
+        <f>B24+C24</f>
+        <v>1218.9293167246526</v>
+      </c>
+      <c r="K25" t="s">
+        <v>71</v>
+      </c>
+      <c r="L25">
+        <v>46.221889892405528</v>
+      </c>
+      <c r="M25">
+        <v>46.243127016089062</v>
+      </c>
+      <c r="N25">
+        <v>46.232580870463721</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K26" t="s">
+        <v>63</v>
+      </c>
+      <c r="L26">
+        <v>5.3841194796800016</v>
+      </c>
+      <c r="M26">
+        <v>5.5155923611825912</v>
+      </c>
+      <c r="N26">
+        <v>5.4435182768766763</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K27" t="s">
+        <v>67</v>
+      </c>
+      <c r="L27">
+        <v>3.0296303147805537</v>
+      </c>
+      <c r="M27">
+        <v>3.112817975691188</v>
+      </c>
+      <c r="N27">
+        <v>3.0672134487654747</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K28" t="s">
+        <v>72</v>
+      </c>
+      <c r="L28">
+        <v>0.29107402544791877</v>
+      </c>
+      <c r="M28">
+        <v>0.28796770498141772</v>
+      </c>
+      <c r="N28">
+        <v>0.28956720143051184</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M30" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M31" s="12">
+        <v>0.70399999999999996</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M32" s="12">
+        <v>0.70380627040878718</v>
+      </c>
+    </row>
+    <row r="33" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M33" s="12">
+        <v>0.70166388640963195</v>
+      </c>
+    </row>
+    <row r="34" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M34" s="12">
+        <v>0.70046889896090037</v>
+      </c>
+    </row>
+    <row r="35" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M35" s="24">
+        <v>0.69917394677785549</v>
+      </c>
+    </row>
+    <row r="36" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M36" s="12">
+        <v>0.69804545423270248</v>
+      </c>
+    </row>
+    <row r="37" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M37" s="12">
+        <v>0.6971320441092701</v>
+      </c>
+    </row>
+    <row r="38" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M38" s="12">
+        <v>0.69601338984367045</v>
+      </c>
+    </row>
+    <row r="39" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M39" s="12">
+        <v>0.69539727621518321</v>
+      </c>
+    </row>
+    <row r="40" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M40" s="12">
+        <v>0.69426566744215223</v>
+      </c>
+    </row>
+    <row r="41" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M41" s="12">
+        <v>0.69353731251708994</v>
+      </c>
+    </row>
+    <row r="42" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M42" s="12">
+        <v>0.69299062205044293</v>
+      </c>
+    </row>
+    <row r="43" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M43" s="12">
+        <v>0.69226271374904658</v>
+      </c>
+    </row>
+    <row r="44" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M44" s="12">
+        <v>0.69164775828557135</v>
+      </c>
+    </row>
+    <row r="45" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M45" s="36">
+        <v>0.69104384879900871</v>
+      </c>
+    </row>
+    <row r="46" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M46" s="12">
+        <v>0.690232937402526</v>
+      </c>
+    </row>
+    <row r="47" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M47" s="12">
+        <v>0.68988576586557904</v>
+      </c>
+    </row>
+    <row r="48" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M48" s="12">
+        <v>0.68964035968165227</v>
+      </c>
+    </row>
+    <row r="49" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M49" s="12">
+        <v>0.68920330986458733</v>
+      </c>
+    </row>
+    <row r="50" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M50" s="12">
+        <v>0.68862556359445315</v>
+      </c>
+    </row>
+    <row r="51" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M51" s="12">
+        <v>0.68833907152648766</v>
+      </c>
+    </row>
+    <row r="52" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="M52" s="12">
+        <v>0.68814953473623941</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A79E6B-3469-4108-ADCD-F97E898FA11C}">
   <dimension ref="A1:DK112"/>
@@ -20785,16 +21807,16 @@
         <f t="shared" si="71"/>
         <v>-1.8871371293862869E-2</v>
       </c>
-      <c r="BJ50" s="104" t="s">
+      <c r="BJ50" s="105" t="s">
         <v>135</v>
       </c>
-      <c r="BK50" s="105"/>
-      <c r="BL50" s="105"/>
-      <c r="BQ50" s="104" t="s">
+      <c r="BK50" s="106"/>
+      <c r="BL50" s="106"/>
+      <c r="BQ50" s="105" t="s">
         <v>138</v>
       </c>
-      <c r="BR50" s="105"/>
-      <c r="BS50" s="105"/>
+      <c r="BR50" s="106"/>
+      <c r="BS50" s="106"/>
       <c r="BV50" s="21"/>
       <c r="BZ50" s="14"/>
       <c r="CA50" s="14"/>
@@ -21134,16 +22156,16 @@
       </c>
     </row>
     <row r="64" spans="1:79" x14ac:dyDescent="0.2">
-      <c r="BJ64" s="104" t="s">
+      <c r="BJ64" s="105" t="s">
         <v>136</v>
       </c>
-      <c r="BK64" s="105"/>
-      <c r="BL64" s="105"/>
-      <c r="BP64" s="104" t="s">
+      <c r="BK64" s="106"/>
+      <c r="BL64" s="106"/>
+      <c r="BP64" s="105" t="s">
         <v>137</v>
       </c>
-      <c r="BQ64" s="105"/>
-      <c r="BR64" s="105"/>
+      <c r="BQ64" s="106"/>
+      <c r="BR64" s="106"/>
     </row>
     <row r="65" spans="61:73" ht="15.75" x14ac:dyDescent="0.25">
       <c r="BI65" s="46" t="s">
@@ -21988,6 +23010,1979 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1243B6B-B859-4272-8CAD-F49C36716C55}">
+  <dimension ref="A1:Y23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="17" width="12" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="104" t="s">
+        <v>228</v>
+      </c>
+      <c r="B1" s="104" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" s="104" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="E1" s="104" t="s">
+        <v>232</v>
+      </c>
+      <c r="F1" s="104" t="s">
+        <v>233</v>
+      </c>
+      <c r="G1" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="104" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1" s="104" t="s">
+        <v>236</v>
+      </c>
+      <c r="J1" s="104" t="s">
+        <v>237</v>
+      </c>
+      <c r="K1" s="104" t="s">
+        <v>238</v>
+      </c>
+      <c r="L1" s="104" t="s">
+        <v>239</v>
+      </c>
+      <c r="M1" s="104" t="s">
+        <v>240</v>
+      </c>
+      <c r="N1" s="104" t="s">
+        <v>241</v>
+      </c>
+      <c r="O1" s="104" t="s">
+        <v>242</v>
+      </c>
+      <c r="P1" s="104" t="s">
+        <v>243</v>
+      </c>
+      <c r="Q1" s="104" t="s">
+        <v>244</v>
+      </c>
+      <c r="R1" s="104" t="s">
+        <v>245</v>
+      </c>
+      <c r="S1" s="104" t="s">
+        <v>246</v>
+      </c>
+      <c r="T1" s="104" t="s">
+        <v>247</v>
+      </c>
+      <c r="X1" s="104" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" s="103">
+        <f>'FS No Vp 100'!A2</f>
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <f>'FS No Vp 100'!AP2</f>
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:C23" si="0">0.5*(1-B2^0.666666667)</f>
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <f t="shared" ref="D2:D23" si="1">-3*$Y$10*((1-2*C2)^2.5)*(1+3*(4-$Y$11)*C2/2)*C2</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <f t="shared" ref="E2:E23" si="2">$Y$2+$Y$5*A2</f>
+        <v>230.92</v>
+      </c>
+      <c r="F2">
+        <f t="shared" ref="F2:F23" si="3">$Y$3+$Y$6*A2</f>
+        <v>120.01</v>
+      </c>
+      <c r="G2">
+        <f t="shared" ref="G2:G23" si="4">$Y$4+$Y$7*A2</f>
+        <v>43.36</v>
+      </c>
+      <c r="H2">
+        <f t="shared" ref="H2:H23" si="5">(E2-F2)/2</f>
+        <v>55.454999999999991</v>
+      </c>
+      <c r="I2">
+        <f t="shared" ref="I2:I23" si="6">(E2+2*F2)/3</f>
+        <v>156.97999999999999</v>
+      </c>
+      <c r="J2">
+        <f t="shared" ref="J2:J23" si="7">(1-2*C2)^3.5*($Y$2-$Y$12*C2)+D2*3</f>
+        <v>230.92</v>
+      </c>
+      <c r="K2">
+        <f t="shared" ref="K2:K23" si="8">(1-2*C2)^3.5*($Y$3-$Y$13*C2)+D2*1</f>
+        <v>120.01</v>
+      </c>
+      <c r="L2">
+        <f t="shared" ref="L2:L23" si="9">(1-2*C2)^3.5*($Y$4-$Y$14*C2)+D2*1</f>
+        <v>43.36</v>
+      </c>
+      <c r="M2">
+        <f t="shared" ref="M2:M23" si="10">(J2-K2)/2</f>
+        <v>55.454999999999991</v>
+      </c>
+      <c r="N2">
+        <f t="shared" ref="N2:N23" si="11">(J2+2*K2)/3</f>
+        <v>156.97999999999999</v>
+      </c>
+      <c r="O2">
+        <f>'FS No Vp 100'!AT2</f>
+        <v>239.73960242643551</v>
+      </c>
+      <c r="P2">
+        <f>'FS No Vp 100'!AV2</f>
+        <v>121.94076995584666</v>
+      </c>
+      <c r="Q2">
+        <f>'FS No Vp 100'!AU2</f>
+        <v>46.232580877717901</v>
+      </c>
+      <c r="R2">
+        <f t="shared" ref="R2:R23" si="12">J2-O2</f>
+        <v>-8.8196024264355231</v>
+      </c>
+      <c r="S2">
+        <f t="shared" ref="S2:S23" si="13">K2-P2</f>
+        <v>-1.9307699558466567</v>
+      </c>
+      <c r="T2">
+        <f t="shared" ref="T2:T23" si="14">L2-Q2</f>
+        <v>-2.8725808777179012</v>
+      </c>
+      <c r="X2" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y2">
+        <v>230.92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A3" s="103">
+        <f>'FS No Vp 100'!A3</f>
+        <v>0.12913290811927533</v>
+      </c>
+      <c r="B3">
+        <f>'FS No Vp 100'!AP3</f>
+        <v>1.0008606381371776</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="0"/>
+        <v>-2.8683824504582844E-4</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="1"/>
+        <v>0.13529274928600155</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="2"/>
+        <v>231.6496009308739</v>
+      </c>
+      <c r="F3">
+        <f t="shared" si="3"/>
+        <v>120.47100448198582</v>
+      </c>
+      <c r="G3">
+        <f t="shared" si="4"/>
+        <v>43.383889588002063</v>
+      </c>
+      <c r="H3">
+        <f t="shared" si="5"/>
+        <v>55.589298224444043</v>
+      </c>
+      <c r="I3">
+        <f t="shared" si="6"/>
+        <v>157.53053663161518</v>
+      </c>
+      <c r="J3">
+        <f t="shared" si="7"/>
+        <v>231.68397002353032</v>
+      </c>
+      <c r="K3">
+        <f t="shared" si="8"/>
+        <v>120.4928438430733</v>
+      </c>
+      <c r="L3">
+        <f t="shared" si="9"/>
+        <v>43.384865918149274</v>
+      </c>
+      <c r="M3">
+        <f t="shared" si="10"/>
+        <v>55.595563090228509</v>
+      </c>
+      <c r="N3">
+        <f t="shared" si="11"/>
+        <v>157.55655256989232</v>
+      </c>
+      <c r="O3">
+        <f>'FS No Vp 100'!AT3</f>
+        <v>240.49536399323526</v>
+      </c>
+      <c r="P3">
+        <f>'FS No Vp 100'!AV3</f>
+        <v>122.36670748862443</v>
+      </c>
+      <c r="Q3">
+        <f>'FS No Vp 100'!AU3</f>
+        <v>46.272622612980577</v>
+      </c>
+      <c r="R3">
+        <f t="shared" si="12"/>
+        <v>-8.8113939697049375</v>
+      </c>
+      <c r="S3">
+        <f t="shared" si="13"/>
+        <v>-1.8738636455511255</v>
+      </c>
+      <c r="T3">
+        <f t="shared" si="14"/>
+        <v>-2.8877566948313032</v>
+      </c>
+      <c r="X3" t="s">
+        <v>219</v>
+      </c>
+      <c r="Y3">
+        <v>120.01</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" s="103">
+        <f>'FS No Vp 100'!A4</f>
+        <v>1.635683502844302</v>
+      </c>
+      <c r="B4">
+        <f>'FS No Vp 100'!AP4</f>
+        <v>1.0104078796601745</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>-3.4633028938252375E-3</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="1"/>
+        <v>1.6616681927127543</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="2"/>
+        <v>240.1616117910703</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="3"/>
+        <v>125.84939010515416</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="4"/>
+        <v>43.662601448026194</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="5"/>
+        <v>57.156110842958071</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="6"/>
+        <v>163.95346400045955</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="7"/>
+        <v>240.24461005376637</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="8"/>
+        <v>125.91999259588272</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="9"/>
+        <v>43.643318725065861</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="10"/>
+        <v>57.162308728941824</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="11"/>
+        <v>164.02819841517726</v>
+      </c>
+      <c r="O4">
+        <f>'FS No Vp 100'!AT4</f>
+        <v>248.94927603743506</v>
+      </c>
+      <c r="P4">
+        <f>'FS No Vp 100'!AV4</f>
+        <v>127.14409945968815</v>
+      </c>
+      <c r="Q4">
+        <f>'FS No Vp 100'!AU4</f>
+        <v>46.698725586174838</v>
+      </c>
+      <c r="R4">
+        <f t="shared" si="12"/>
+        <v>-8.7046659836686899</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="13"/>
+        <v>-1.2241068638054315</v>
+      </c>
+      <c r="T4">
+        <f t="shared" si="14"/>
+        <v>-3.0554068611089775</v>
+      </c>
+      <c r="X4" t="s">
+        <v>220</v>
+      </c>
+      <c r="Y4">
+        <v>43.36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A5" s="103">
+        <f>'FS No Vp 100'!A5</f>
+        <v>2.4965695569728967</v>
+      </c>
+      <c r="B5">
+        <f>'FS No Vp 100'!AP5</f>
+        <v>1.0157208218118636</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>-5.2266387673991499E-3</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="1"/>
+        <v>2.5314790847860875</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="2"/>
+        <v>245.02561799689687</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="3"/>
+        <v>128.92275331839323</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="4"/>
+        <v>43.821865368039987</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="5"/>
+        <v>58.051432339251818</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="6"/>
+        <v>167.62370821122778</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="7"/>
+        <v>245.0768250744477</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="8"/>
+        <v>128.99676482088827</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="9"/>
+        <v>43.773086426318763</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="10"/>
+        <v>58.040030126779712</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="11"/>
+        <v>167.69011823874141</v>
+      </c>
+      <c r="O5">
+        <f>'FS No Vp 100'!AT5</f>
+        <v>253.70942977356148</v>
+      </c>
+      <c r="P5">
+        <f>'FS No Vp 100'!AV5</f>
+        <v>129.84443704444371</v>
+      </c>
+      <c r="Q5">
+        <f>'FS No Vp 100'!AU5</f>
+        <v>46.921193614301146</v>
+      </c>
+      <c r="R5">
+        <f t="shared" si="12"/>
+        <v>-8.6326046991137844</v>
+      </c>
+      <c r="S5">
+        <f t="shared" si="13"/>
+        <v>-0.84767222355543481</v>
+      </c>
+      <c r="T5">
+        <f t="shared" si="14"/>
+        <v>-3.148107187982383</v>
+      </c>
+      <c r="X5" t="s">
+        <v>221</v>
+      </c>
+      <c r="Y5">
+        <v>5.65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="103">
+        <f>'FS No Vp 100'!A6</f>
+        <v>3.4435442165143506</v>
+      </c>
+      <c r="B6">
+        <f>'FS No Vp 100'!AP6</f>
+        <v>1.0214600339474598</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>-7.1280004971914224E-3</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="1"/>
+        <v>3.4875731842468998</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="2"/>
+        <v>250.37602482330607</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="3"/>
+        <v>132.30345285295624</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="4"/>
+        <v>43.997055680055155</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="5"/>
+        <v>59.036285985174914</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="6"/>
+        <v>171.66097684307283</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="7"/>
+        <v>250.3517939971577</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="8"/>
+        <v>132.36621774689917</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="9"/>
+        <v>43.901716115775095</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="10"/>
+        <v>58.992788125129266</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="11"/>
+        <v>171.69474316365199</v>
+      </c>
+      <c r="O6">
+        <f>'FS No Vp 100'!AT6</f>
+        <v>258.89614801271489</v>
+      </c>
+      <c r="P6">
+        <f>'FS No Vp 100'!AV6</f>
+        <v>132.79514599272454</v>
+      </c>
+      <c r="Q6">
+        <f>'FS No Vp 100'!AU6</f>
+        <v>47.149440291484936</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="12"/>
+        <v>-8.5443540155571895</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="13"/>
+        <v>-0.42892824582537514</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="14"/>
+        <v>-3.2477241757098412</v>
+      </c>
+      <c r="X6" t="s">
+        <v>222</v>
+      </c>
+      <c r="Y6">
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="103">
+        <f>'FS No Vp 100'!A7</f>
+        <v>4.4335631787622765</v>
+      </c>
+      <c r="B7">
+        <f>'FS No Vp 100'!AP7</f>
+        <v>1.0273540898824036</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>-9.076958183110384E-3</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="1"/>
+        <v>4.4873902342069272</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="2"/>
+        <v>255.96963196000684</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="3"/>
+        <v>135.83782054818133</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="4"/>
+        <v>44.180209188071018</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="5"/>
+        <v>60.065905705912755</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="6"/>
+        <v>175.88175768545648</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="7"/>
+        <v>255.82874822596364</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="8"/>
+        <v>135.87641080493881</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="9"/>
+        <v>44.021104351806436</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="10"/>
+        <v>59.976168710512411</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="11"/>
+        <v>175.86052327861375</v>
+      </c>
+      <c r="O7">
+        <f>'FS No Vp 100'!AT7</f>
+        <v>264.27101498123528</v>
+      </c>
+      <c r="P7">
+        <f>'FS No Vp 100'!AV7</f>
+        <v>135.86205392458635</v>
+      </c>
+      <c r="Q7">
+        <f>'FS No Vp 100'!AU7</f>
+        <v>47.370531986943298</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="12"/>
+        <v>-8.4422667552716462</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="13"/>
+        <v>1.4356880352465851E-2</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="14"/>
+        <v>-3.3494276351368626</v>
+      </c>
+      <c r="X7" t="s">
+        <v>223</v>
+      </c>
+      <c r="Y7">
+        <v>0.185</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A8" s="103">
+        <f>'FS No Vp 100'!A8</f>
+        <v>5.1222720220651237</v>
+      </c>
+      <c r="B8">
+        <f>'FS No Vp 100'!AP8</f>
+        <v>1.0313936004615611</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>-1.0410530513957128E-2</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="1"/>
+        <v>5.1831612632296871</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="2"/>
+        <v>259.86083692466792</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="3"/>
+        <v>138.29651111877249</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="4"/>
+        <v>44.307620324082045</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="5"/>
+        <v>60.782162902947718</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="6"/>
+        <v>178.81795305407095</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="7"/>
+        <v>259.61739822857953</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="8"/>
+        <v>138.31145701466136</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="9"/>
+        <v>44.095365120883351</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="10"/>
+        <v>60.652970606959087</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="11"/>
+        <v>178.74677075263409</v>
+      </c>
+      <c r="O8">
+        <f>'FS No Vp 100'!AT8</f>
+        <v>267.98288390863308</v>
+      </c>
+      <c r="P8">
+        <f>'FS No Vp 100'!AV8</f>
+        <v>137.98545838593489</v>
+      </c>
+      <c r="Q8">
+        <f>'FS No Vp 100'!AU8</f>
+        <v>47.514123031050097</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="12"/>
+        <v>-8.3654856800535526</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="13"/>
+        <v>0.32599862872646668</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="14"/>
+        <v>-3.4187579101667467</v>
+      </c>
+      <c r="X8" t="s">
+        <v>224</v>
+      </c>
+      <c r="Y8">
+        <f>(Y2-Y3)/2</f>
+        <v>55.454999999999991</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A9" s="103">
+        <f>'FS No Vp 100'!A9</f>
+        <v>5.7679365626615837</v>
+      </c>
+      <c r="B9">
+        <f>'FS No Vp 100'!AP9</f>
+        <v>1.0351406911514562</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-1.1646009933598656E-2</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="1"/>
+        <v>5.8362643253649731</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="2"/>
+        <v>263.50884157903795</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="3"/>
+        <v>140.60153352870185</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="4"/>
+        <v>44.427068264092391</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="5"/>
+        <v>61.453654025168049</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="6"/>
+        <v>181.57063621214721</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="7"/>
+        <v>263.15729113429251</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="8"/>
+        <v>140.59165465543859</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="9"/>
+        <v>44.158673106297172</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="10"/>
+        <v>61.282818239426959</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="11"/>
+        <v>181.44686681505655</v>
+      </c>
+      <c r="O9">
+        <f>'FS No Vp 100'!AT9</f>
+        <v>271.44652765662096</v>
+      </c>
+      <c r="P9">
+        <f>'FS No Vp 100'!AV9</f>
+        <v>139.97082339632456</v>
+      </c>
+      <c r="Q9">
+        <f>'FS No Vp 100'!AU9</f>
+        <v>47.641458428112784</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="12"/>
+        <v>-8.2892365223284514</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="13"/>
+        <v>0.62083125911402703</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="14"/>
+        <v>-3.4827853218156122</v>
+      </c>
+      <c r="X9" t="s">
+        <v>225</v>
+      </c>
+      <c r="Y9">
+        <f>(Y5-Y6)/2</f>
+        <v>1.0400000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A10" s="103">
+        <f>'FS No Vp 100'!A10</f>
+        <v>6.5857783140837629</v>
+      </c>
+      <c r="B10">
+        <f>'FS No Vp 100'!AP10</f>
+        <v>1.0398336989916428</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>-1.3191273652871427E-2</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="1"/>
+        <v>6.664729006027903</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="2"/>
+        <v>268.12964747457323</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="3"/>
+        <v>143.52122858127905</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="4"/>
+        <v>44.578368988105495</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="5"/>
+        <v>62.304209446647093</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="6"/>
+        <v>185.0573682123771</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="7"/>
+        <v>267.62548265207175</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="8"/>
+        <v>143.47667738212618</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="9"/>
+        <v>44.230294329815273</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="10"/>
+        <v>62.074402634972785</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="11"/>
+        <v>184.85961247210807</v>
+      </c>
+      <c r="O10">
+        <f>'FS No Vp 100'!AT10</f>
+        <v>275.81231046183507</v>
+      </c>
+      <c r="P10">
+        <f>'FS No Vp 100'!AV10</f>
+        <v>142.47871246948213</v>
+      </c>
+      <c r="Q10">
+        <f>'FS No Vp 100'!AU10</f>
+        <v>47.792868189067008</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="12"/>
+        <v>-8.1868278097633151</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="13"/>
+        <v>0.99796491264405063</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="14"/>
+        <v>-3.5625738592517351</v>
+      </c>
+      <c r="X10" t="s">
+        <v>226</v>
+      </c>
+      <c r="Y10">
+        <f>(Y2+2*Y3)/3</f>
+        <v>156.97999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A11" s="103">
+        <f>'FS No Vp 100'!A11</f>
+        <v>7.274487157386611</v>
+      </c>
+      <c r="B11">
+        <f>'FS No Vp 100'!AP11</f>
+        <v>1.043737266686328</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>-1.4474828624401415E-2</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="1"/>
+        <v>7.3627551646404727</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="2"/>
+        <v>272.02085243923432</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="3"/>
+        <v>145.97991915187021</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="4"/>
+        <v>44.705780124116522</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="5"/>
+        <v>63.020466643682056</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="6"/>
+        <v>187.99356358099158</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="7"/>
+        <v>271.37149253624949</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="8"/>
+        <v>145.90124610223714</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="9"/>
+        <v>44.28328961431572</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="10"/>
+        <v>62.735123217006176</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="11"/>
+        <v>187.72466158024125</v>
+      </c>
+      <c r="O11">
+        <f>'FS No Vp 100'!AT11</f>
+        <v>279.46720957325931</v>
+      </c>
+      <c r="P11">
+        <f>'FS No Vp 100'!AV11</f>
+        <v>144.58286133502438</v>
+      </c>
+      <c r="Q11">
+        <f>'FS No Vp 100'!AU11</f>
+        <v>47.911875969788625</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="12"/>
+        <v>-8.0957170370098197</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="13"/>
+        <v>1.3183847672127627</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="14"/>
+        <v>-3.6285863554729048</v>
+      </c>
+      <c r="X11" t="s">
+        <v>227</v>
+      </c>
+      <c r="Y11">
+        <f>(Y5+2*Y6)/3</f>
+        <v>4.2633333333333328</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A12" s="103">
+        <f>'FS No Vp 100'!A12</f>
+        <v>7.834063092570239</v>
+      </c>
+      <c r="B12">
+        <f>'FS No Vp 100'!AP12</f>
+        <v>1.0468790795775158</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>-1.5506744641379022E-2</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="1"/>
+        <v>7.9304730650281074</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="2"/>
+        <v>275.18245647302183</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="3"/>
+        <v>147.97760524047575</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="4"/>
+        <v>44.809301672125493</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="5"/>
+        <v>63.602425616273038</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="6"/>
+        <v>190.37922231799112</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="7"/>
+        <v>274.40594766044376</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="8"/>
+        <v>147.86913721474087</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="9"/>
+        <v>44.321552956577008</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="10"/>
+        <v>63.268405222851442</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="11"/>
+        <v>190.04807402997517</v>
+      </c>
+      <c r="O12">
+        <f>'FS No Vp 100'!AT12</f>
+        <v>282.42437644804556</v>
+      </c>
+      <c r="P12">
+        <f>'FS No Vp 100'!AV12</f>
+        <v>146.28838849945876</v>
+      </c>
+      <c r="Q12">
+        <f>'FS No Vp 100'!AU12</f>
+        <v>48.003027553979706</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="12"/>
+        <v>-8.0184287876018061</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="13"/>
+        <v>1.5807487152821125</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="14"/>
+        <v>-3.6814745974026977</v>
+      </c>
+      <c r="X12" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y12">
+        <f>3*Y10*(Y5-3)-7*Y2</f>
+        <v>-368.44899999999984</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A13" s="103">
+        <f>'FS No Vp 100'!A13</f>
+        <v>8.5227719358730862</v>
+      </c>
+      <c r="B13">
+        <f>'FS No Vp 100'!AP13</f>
+        <v>1.0507114083996756</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>-1.6764061431739696E-2</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="1"/>
+        <v>8.6301213551604814</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="2"/>
+        <v>279.07366143768292</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="3"/>
+        <v>150.43629581106691</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="4"/>
+        <v>44.936712808136519</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="5"/>
+        <v>64.318682813308001</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="6"/>
+        <v>193.31541768660557</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="7"/>
+        <v>278.13085039196034</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="8"/>
+        <v>150.28948622834534</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="9"/>
+        <v>44.362867523835121</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="10"/>
+        <v>63.920682081807499</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="11"/>
+        <v>192.90327428288367</v>
+      </c>
+      <c r="O13">
+        <f>'FS No Vp 100'!AT13</f>
+        <v>286.05017440501143</v>
+      </c>
+      <c r="P13">
+        <f>'FS No Vp 100'!AV13</f>
+        <v>148.38327169385553</v>
+      </c>
+      <c r="Q13">
+        <f>'FS No Vp 100'!AU13</f>
+        <v>48.10855193910696</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="12"/>
+        <v>-7.9193240130510958</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="13"/>
+        <v>1.9062145344898056</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="14"/>
+        <v>-3.7456844152718389</v>
+      </c>
+      <c r="X13" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y13">
+        <f>3*Y10*(Y6-1)-7*Y3</f>
+        <v>370.2457999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A14" s="103">
+        <f>'FS No Vp 100'!A14</f>
+        <v>9.1253921737631298</v>
+      </c>
+      <c r="B14">
+        <f>'FS No Vp 100'!AP14</f>
+        <v>1.0540320452210339</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>-1.7852265840293979E-2</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="1"/>
+        <v>9.2427319728542141</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="2"/>
+        <v>282.47846578176166</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="3"/>
+        <v>152.58765006033437</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="4"/>
+        <v>45.048197552146178</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="5"/>
+        <v>64.945407860713644</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="6"/>
+        <v>195.88458863414348</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="7"/>
+        <v>281.37934466201739</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="8"/>
+        <v>152.4044622257947</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="9"/>
+        <v>44.393855475420651</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="10"/>
+        <v>64.487441218111343</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="11"/>
+        <v>195.3960897045356</v>
+      </c>
+      <c r="O14">
+        <f>'FS No Vp 100'!AT14</f>
+        <v>289.20846032771999</v>
+      </c>
+      <c r="P14">
+        <f>'FS No Vp 100'!AV14</f>
+        <v>150.21137147232668</v>
+      </c>
+      <c r="Q14">
+        <f>'FS No Vp 100'!AU14</f>
+        <v>48.194899555122817</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="12"/>
+        <v>-7.8291156657026022</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="13"/>
+        <v>2.1930907534680273</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="14"/>
+        <v>-3.8010440797021658</v>
+      </c>
+      <c r="X14" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y14">
+        <f>3*Y10*(Y7-1)-7*Y4</f>
+        <v>-687.33609999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A15" s="103">
+        <f>'FS No Vp 100'!A15</f>
+        <v>9.5558352008274561</v>
+      </c>
+      <c r="B15">
+        <f>'FS No Vp 100'!AP15</f>
+        <v>1.0563870694672328</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>-1.8623337242798632E-2</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="1"/>
+        <v>9.6808008630940439</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="2"/>
+        <v>284.91046888467514</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="3"/>
+        <v>154.12433166695402</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="4"/>
+        <v>45.127829512153077</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="5"/>
+        <v>65.39306860886056</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="6"/>
+        <v>197.71971073952773</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="7"/>
+        <v>283.69500484983877</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="8"/>
+        <v>153.91446587994776</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="9"/>
+        <v>44.413100334884312</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="10"/>
+        <v>64.890269484945506</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="11"/>
+        <v>197.17464553657808</v>
+      </c>
+      <c r="O15">
+        <f>'FS No Vp 100'!AT15</f>
+        <v>291.45768120022001</v>
+      </c>
+      <c r="P15">
+        <f>'FS No Vp 100'!AV15</f>
+        <v>151.5151642562343</v>
+      </c>
+      <c r="Q15">
+        <f>'FS No Vp 100'!AU15</f>
+        <v>48.253245903837538</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="12"/>
+        <v>-7.7626763503812413</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="13"/>
+        <v>2.3993016237134555</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="14"/>
+        <v>-3.8401455689532256</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A16" s="103">
+        <f>'FS No Vp 100'!A16</f>
+        <v>10.115411136011028</v>
+      </c>
+      <c r="B16">
+        <f>'FS No Vp 100'!AP16</f>
+        <v>1.0594304379273183</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>-1.961893507883794E-2</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="1"/>
+        <v>10.251348608444646</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="2"/>
+        <v>288.07207291846231</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="3"/>
+        <v>156.12201775555937</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="4"/>
+        <v>45.231351060162041</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="5"/>
+        <v>65.975027581451471</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="6"/>
+        <v>200.10536947652702</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="7"/>
+        <v>286.70202613803133</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="8"/>
+        <v>155.87820755629454</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="9"/>
+        <v>44.434583730428784</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="10"/>
+        <v>65.411909290868394</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="11"/>
+        <v>199.48614708354012</v>
+      </c>
+      <c r="O16">
+        <f>'FS No Vp 100'!AT16</f>
+        <v>294.37579098479722</v>
+      </c>
+      <c r="P16">
+        <f>'FS No Vp 100'!AV16</f>
+        <v>153.20901550110361</v>
+      </c>
+      <c r="Q16">
+        <f>'FS No Vp 100'!AU16</f>
+        <v>48.325058115880026</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="12"/>
+        <v>-7.6737648467658914</v>
+      </c>
+      <c r="S16">
+        <f t="shared" si="13"/>
+        <v>2.6691920551909334</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="14"/>
+        <v>-3.8904743854512418</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A17" s="103">
+        <f>'FS No Vp 100'!A17</f>
+        <v>10.631942768488157</v>
+      </c>
+      <c r="B17">
+        <f>'FS No Vp 100'!AP17</f>
+        <v>1.0622184453754944</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>-2.0530158537102716E-2</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="1"/>
+        <v>10.778424485744049</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="2"/>
+        <v>290.99047664195808</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="3"/>
+        <v>157.96603568350272</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="4"/>
+        <v>45.326909412170309</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="5"/>
+        <v>66.512220479227679</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="6"/>
+        <v>202.30751600298785</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="7"/>
+        <v>289.47112426669025</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="8"/>
+        <v>157.68946445489158</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="9"/>
+        <v>44.450886960482364</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="10"/>
+        <v>65.890829905899338</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="11"/>
+        <v>201.61668439215782</v>
+      </c>
+      <c r="O17">
+        <f>'FS No Vp 100'!AT17</f>
+        <v>297.06039310509186</v>
+      </c>
+      <c r="P17">
+        <f>'FS No Vp 100'!AV17</f>
+        <v>154.7696385585584</v>
+      </c>
+      <c r="Q17">
+        <f>'FS No Vp 100'!AU17</f>
+        <v>48.387263279956642</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="12"/>
+        <v>-7.5892688384016083</v>
+      </c>
+      <c r="S17">
+        <f t="shared" si="13"/>
+        <v>2.9198258963331796</v>
+      </c>
+      <c r="T17">
+        <f t="shared" si="14"/>
+        <v>-3.9363763194742774</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A18" s="103">
+        <f>'FS No Vp 100'!A18</f>
+        <v>10.933252887433179</v>
+      </c>
+      <c r="B18">
+        <f>'FS No Vp 100'!AP18</f>
+        <v>1.0638338109366763</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>-2.1057754670470885E-2</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="1"/>
+        <v>11.085741034064565</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="2"/>
+        <v>292.69287881399748</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="3"/>
+        <v>159.04171280813645</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="4"/>
+        <v>45.382651784175138</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="5"/>
+        <v>66.825583002930514</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="6"/>
+        <v>203.59210147675677</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="7"/>
+        <v>291.08183553908111</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="8"/>
+        <v>158.74429234494102</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="9"/>
+        <v>44.458844786033197</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="10"/>
+        <v>66.168771597070048</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="11"/>
+        <v>202.85680674298771</v>
+      </c>
+      <c r="O18">
+        <f>'FS No Vp 100'!AT18</f>
+        <v>298.62080590430099</v>
+      </c>
+      <c r="P18">
+        <f>'FS No Vp 100'!AV18</f>
+        <v>155.67775972928965</v>
+      </c>
+      <c r="Q18">
+        <f>'FS No Vp 100'!AU18</f>
+        <v>48.42172558418833</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="12"/>
+        <v>-7.5389703652198818</v>
+      </c>
+      <c r="S18">
+        <f t="shared" si="13"/>
+        <v>3.0665326156513686</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="14"/>
+        <v>-3.9628807981551333</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A19" s="103">
+        <f>'FS No Vp 100'!A19</f>
+        <v>11.148474400965315</v>
+      </c>
+      <c r="B19">
+        <f>'FS No Vp 100'!AP19</f>
+        <v>1.0649827168712658</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>-2.1432837469644528E-2</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="1"/>
+        <v>11.305178694317265</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="2"/>
+        <v>293.90888036545402</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="3"/>
+        <v>159.81005361144616</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="4"/>
+        <v>45.422467764178585</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="5"/>
+        <v>67.04941337700393</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="6"/>
+        <v>204.50966252944878</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="7"/>
+        <v>292.2302470642407</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="8"/>
+        <v>159.49693462731557</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="9"/>
+        <v>44.463836700504302</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="10"/>
+        <v>66.366656218462566</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="11"/>
+        <v>203.74137210629064</v>
+      </c>
+      <c r="O19">
+        <f>'FS No Vp 100'!AT19</f>
+        <v>299.73284114549477</v>
+      </c>
+      <c r="P19">
+        <f>'FS No Vp 100'!AV19</f>
+        <v>156.3253912680116</v>
+      </c>
+      <c r="Q19">
+        <f>'FS No Vp 100'!AU19</f>
+        <v>48.445527207891473</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="12"/>
+        <v>-7.5025940812540739</v>
+      </c>
+      <c r="S19">
+        <f t="shared" si="13"/>
+        <v>3.1715433593039677</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="14"/>
+        <v>-3.9816905073871709</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20" s="103">
+        <f>'FS No Vp 100'!A20</f>
+        <v>11.535873125323196</v>
+      </c>
+      <c r="B20">
+        <f>'FS No Vp 100'!AP20</f>
+        <v>1.0670419517105312</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>-2.2104777595228886E-2</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="1"/>
+        <v>11.700284468529668</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="2"/>
+        <v>296.09768315807605</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="3"/>
+        <v>161.19306705740382</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="4"/>
+        <v>45.494136528184789</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="5"/>
+        <v>67.452308050336114</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="6"/>
+        <v>206.16127242429457</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="7"/>
+        <v>294.29445726548329</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="8"/>
+        <v>160.85095167458007</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="9"/>
+        <v>44.471388109415528</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="10"/>
+        <v>66.721752795451607</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="11"/>
+        <v>205.33212020488114</v>
+      </c>
+      <c r="O20">
+        <f>'FS No Vp 100'!AT20</f>
+        <v>301.73059411971252</v>
+      </c>
+      <c r="P20">
+        <f>'FS No Vp 100'!AV20</f>
+        <v>157.48979975987265</v>
+      </c>
+      <c r="Q20">
+        <f>'FS No Vp 100'!AU20</f>
+        <v>48.486705255422322</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="12"/>
+        <v>-7.4361368542292325</v>
+      </c>
+      <c r="S20">
+        <f t="shared" si="13"/>
+        <v>3.3611519147074205</v>
+      </c>
+      <c r="T20">
+        <f t="shared" si="14"/>
+        <v>-4.0153171460067938</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21" s="103">
+        <f>'FS No Vp 100'!A21</f>
+        <v>12.052404757800351</v>
+      </c>
+      <c r="B21">
+        <f>'FS No Vp 100'!AP21</f>
+        <v>1.0697685400291816</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>-2.2993814311138894E-2</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="1"/>
+        <v>12.226993127334094</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="2"/>
+        <v>299.01608688157199</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="3"/>
+        <v>163.03708498534726</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="4"/>
+        <v>45.589694880193065</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="5"/>
+        <v>67.989500948112365</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="6"/>
+        <v>208.36341895075552</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="7"/>
+        <v>297.03922100034822</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="8"/>
+        <v>162.65371778585973</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="9"/>
+        <v>44.478614312288315</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="10"/>
+        <v>67.192751607244247</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="11"/>
+        <v>207.44888552402256</v>
+      </c>
+      <c r="O21">
+        <f>'FS No Vp 100'!AT21</f>
+        <v>304.38486370085593</v>
+      </c>
+      <c r="P21">
+        <f>'FS No Vp 100'!AV21</f>
+        <v>159.03874695125342</v>
+      </c>
+      <c r="Q21">
+        <f>'FS No Vp 100'!AU21</f>
+        <v>48.538281628821721</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="12"/>
+        <v>-7.3456427005077103</v>
+      </c>
+      <c r="S21">
+        <f t="shared" si="13"/>
+        <v>3.6149708346063107</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="14"/>
+        <v>-4.0596673165334067</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A22" s="103">
+        <f>'FS No Vp 100'!A22</f>
+        <v>12.31067057403893</v>
+      </c>
+      <c r="B22">
+        <f>'FS No Vp 100'!AP22</f>
+        <v>1.0711217084948135</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>-2.3434750581144526E-2</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="1"/>
+        <v>12.489899288644324</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="2"/>
+        <v>300.47528874331994</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="3"/>
+        <v>163.95909394931897</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="4"/>
+        <v>45.637474056197199</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="5"/>
+        <v>68.258097397000483</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="6"/>
+        <v>209.46449221398598</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="7"/>
+        <v>298.4063163297219</v>
+      </c>
+      <c r="K22">
+        <f t="shared" si="8"/>
+        <v>163.55262047372761</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="9"/>
+        <v>44.481020900796437</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="10"/>
+        <v>67.426847927997144</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="11"/>
+        <v>208.50385242572574</v>
+      </c>
+      <c r="O22">
+        <f>'FS No Vp 100'!AT22</f>
+        <v>305.70598442612572</v>
+      </c>
+      <c r="P22">
+        <f>'FS No Vp 100'!AV22</f>
+        <v>159.81050952334911</v>
+      </c>
+      <c r="Q22">
+        <f>'FS No Vp 100'!AU22</f>
+        <v>48.562623782323286</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="12"/>
+        <v>-7.2996680964038205</v>
+      </c>
+      <c r="S22">
+        <f t="shared" si="13"/>
+        <v>3.7421109503785033</v>
+      </c>
+      <c r="T22">
+        <f t="shared" si="14"/>
+        <v>-4.0816028815268481</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A23" s="103">
+        <f>'FS No Vp 100'!A23</f>
+        <v>12.482847784864649</v>
+      </c>
+      <c r="B23">
+        <f>'FS No Vp 100'!AP23</f>
+        <v>1.0720197558999069</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>-2.3727281022046576E-2</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="1"/>
+        <v>12.664933301816427</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="2"/>
+        <v>301.44808998448525</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="3"/>
+        <v>164.5737665919668</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="4"/>
+        <v>45.669326840199957</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="5"/>
+        <v>68.437161696259224</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="6"/>
+        <v>210.19854105613959</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="7"/>
+        <v>299.31540461300176</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="8"/>
+        <v>164.15073461091487</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="9"/>
+        <v>44.482184051264248</v>
+      </c>
+      <c r="M23">
+        <f t="shared" si="10"/>
+        <v>67.582335001043447</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="11"/>
+        <v>209.20562461161049</v>
+      </c>
+      <c r="O23">
+        <f>'FS No Vp 100'!AT23</f>
+        <v>306.58416976799867</v>
+      </c>
+      <c r="P23">
+        <f>'FS No Vp 100'!AV23</f>
+        <v>160.32381448327351</v>
+      </c>
+      <c r="Q23">
+        <f>'FS No Vp 100'!AU23</f>
+        <v>48.578317008639431</v>
+      </c>
+      <c r="R23">
+        <f t="shared" si="12"/>
+        <v>-7.2687651549969132</v>
+      </c>
+      <c r="S23">
+        <f t="shared" si="13"/>
+        <v>3.8269201276413582</v>
+      </c>
+      <c r="T23">
+        <f t="shared" si="14"/>
+        <v>-4.0961329573751826</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDBE080D-85DE-465C-A46B-D92EB166E59B}">
   <dimension ref="A1:EJ112"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -31833,7 +34828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A67F0C9-C9E8-4466-B2F6-2987585B8340}">
   <dimension ref="A1:EH112"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -41659,7 +44654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4544543-076C-4BEB-BE9F-817032EFE3FB}">
   <dimension ref="A1:EK112"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -51634,7 +54629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:S52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -52553,923 +55548,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12A38178-9331-4F70-84AF-90930ECA28C5}">
-  <dimension ref="A1:S52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="15" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D3" t="s">
-        <v>160</v>
-      </c>
-      <c r="E3" t="s">
-        <v>161</v>
-      </c>
-      <c r="F3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G3" t="s">
-        <v>163</v>
-      </c>
-      <c r="H3" t="s">
-        <v>164</v>
-      </c>
-      <c r="I3" t="s">
-        <v>165</v>
-      </c>
-      <c r="J3" t="s">
-        <v>166</v>
-      </c>
-      <c r="K3" t="s">
-        <v>167</v>
-      </c>
-      <c r="L3" t="s">
-        <v>168</v>
-      </c>
-      <c r="M3" t="s">
-        <v>169</v>
-      </c>
-      <c r="N3" t="s">
-        <v>170</v>
-      </c>
-      <c r="O3" t="s">
-        <v>171</v>
-      </c>
-      <c r="P3" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>173</v>
-      </c>
-      <c r="S3" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="103">
-        <f>'FS No Vs 111'!BG25</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="C4" s="103">
-        <f>'FS No Vp 111'!BC25</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="D4" s="103">
-        <f>'FS No Vs 100'!BF25</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="E4" s="103">
-        <f>'FS No Vp 100'!BH25</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="F4" s="103">
-        <f>'FS No Vs 111'!AP26</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="G4" s="103">
-        <f>'FS No Vp 111'!AQ28</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="H4" s="103">
-        <f>'FS No Vs 100'!AQ26</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="I4" s="103">
-        <f>'FS No Vp 100'!AS26</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <f t="shared" ref="K4:K9" si="0">AVERAGE(B4:E4)</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="L4">
-        <f t="shared" ref="L4:L9" si="1">AVERAGE(F4:I4)</f>
-        <v>239.73960242643551</v>
-      </c>
-      <c r="M4">
-        <f t="shared" ref="M4:M9" si="2">AVERAGE(B4:I4)</f>
-        <v>239.73960242643554</v>
-      </c>
-      <c r="N4">
-        <f t="shared" ref="N4:N9" si="3">J4*IF($D$11=1,DEVSQ(B4:E4)/K4^2,DEVSQ(B4:E4))</f>
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <f t="shared" ref="O4:O9" si="4">J4*IF($D$11=1,DEVSQ(F4:I4)/L4^2,DEVSQ(F4:I4))</f>
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <f t="shared" ref="P4:P9" si="5">J4*IF($D$11=1,(K4-L4)^2/M4^2,(K4-L4)^2)</f>
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <f t="shared" ref="Q4:Q9" si="6">J4*IF($D$11=1,DEVSQ(B4:I4)/M4^2,DEVSQ(B4:I4))</f>
-        <v>6.4623485355705287E-27</v>
-      </c>
-      <c r="S4" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="103">
-        <f>'FS No Vs 111'!BG26</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="C5" s="103">
-        <f>'FS No Vp 111'!BC26</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="D5" s="103">
-        <f>'FS No Vs 100'!BF26</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="E5" s="103">
-        <f>'FS No Vp 100'!BH26</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="F5" s="103">
-        <f>'FS No Vs 111'!AP27</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="G5" s="103">
-        <f>'FS No Vp 111'!AQ29</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="H5" s="103">
-        <f>'FS No Vs 100'!AQ27</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="I5" s="103">
-        <f>'FS No Vp 100'!AS27</f>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <f t="shared" si="0"/>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="L5">
-        <f t="shared" si="1"/>
-        <v>121.94076995584666</v>
-      </c>
-      <c r="M5">
-        <f t="shared" si="2"/>
-        <v>121.94076995584668</v>
-      </c>
-      <c r="N5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <f t="shared" si="6"/>
-        <v>1.6155871338926322E-27</v>
-      </c>
-      <c r="S5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="103">
-        <f>'FS No Vs 111'!BG27</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="C6" s="103">
-        <f>'FS No Vp 111'!BC27</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="D6" s="103">
-        <f>'FS No Vs 100'!BF27</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="E6" s="103">
-        <f>'FS No Vp 100'!BH27</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="F6" s="103">
-        <f>'FS No Vs 111'!AP28</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="G6" s="103">
-        <f>'FS No Vp 111'!AQ30</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="H6" s="103">
-        <f>'FS No Vs 100'!AQ28</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="I6" s="103">
-        <f>'FS No Vp 100'!AS28</f>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <f t="shared" si="0"/>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="L6">
-        <f t="shared" si="1"/>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="M6">
-        <f t="shared" si="2"/>
-        <v>46.232580877717901</v>
-      </c>
-      <c r="N6">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="S6" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="103">
-        <f>'FS No Vs 111'!BG28</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="C7" s="103">
-        <f>'FS No Vp 111'!BC28</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="D7" s="103">
-        <f>'FS No Vs 100'!BF28</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="E7" s="103">
-        <f>'FS No Vp 100'!BH28</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="F7" s="103">
-        <f>'FS No Vs 111'!AR26</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="G7" s="103">
-        <f>'FS No Vp 111'!AQ31</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="H7" s="103">
-        <f>'FS No Vs 100'!AQ29</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="I7" s="103">
-        <f>'FS No Vp 100'!AS29</f>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <f t="shared" si="0"/>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="L7">
-        <f t="shared" si="1"/>
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="M7">
-        <f t="shared" si="2"/>
-        <v>5.4435182877526822</v>
-      </c>
-      <c r="N7">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O7">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="S7" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="103">
-        <f>'FS No Vs 111'!BG29</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="C8" s="103">
-        <f>'FS No Vp 111'!BC29</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="D8" s="103">
-        <f>'FS No Vs 100'!BF29</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="E8" s="103">
-        <f>'FS No Vp 100'!BH29</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="F8" s="103">
-        <f>'FS No Vs 111'!AR27</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="G8" s="103">
-        <f>'FS No Vp 111'!AQ32</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="H8" s="103">
-        <f>'FS No Vs 100'!AQ30</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="I8" s="103">
-        <f>'FS No Vp 100'!AS30</f>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <f t="shared" si="0"/>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="L8">
-        <f t="shared" si="1"/>
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="M8">
-        <f t="shared" si="2"/>
-        <v>3.0672134474127288</v>
-      </c>
-      <c r="N8">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q8">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="S8" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="103">
-        <f>'FS No Vs 111'!BG30</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="C9" s="103">
-        <f>'FS No Vp 111'!BC30</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="D9" s="103">
-        <f>'FS No Vs 100'!BF30</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="E9" s="103">
-        <f>'FS No Vp 100'!BH30</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="F9" s="103">
-        <f>'FS No Vs 111'!AR28</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="G9" s="103">
-        <f>'FS No Vp 111'!AQ33</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="H9" s="103">
-        <f>'FS No Vs 100'!AQ31</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="I9" s="103">
-        <f>'FS No Vp 100'!AS31</f>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <f t="shared" si="0"/>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="L9">
-        <f t="shared" si="1"/>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="M9">
-        <f t="shared" si="2"/>
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="N9">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="O9">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q9">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="S9" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>181</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="L11" t="s">
-        <v>203</v>
-      </c>
-      <c r="M11" t="s">
-        <v>205</v>
-      </c>
-      <c r="S11" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="K12" t="s">
-        <v>62</v>
-      </c>
-      <c r="L12">
-        <v>239.73960242643551</v>
-      </c>
-      <c r="M12">
-        <v>239.510382116199</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>183</v>
-      </c>
-      <c r="E13">
-        <f>SUM(N4:N9)</f>
-        <v>0</v>
-      </c>
-      <c r="K13" t="s">
-        <v>66</v>
-      </c>
-      <c r="L13">
-        <v>121.94076995584666</v>
-      </c>
-      <c r="M13">
-        <v>121.79137881717247</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>184</v>
-      </c>
-      <c r="E14">
-        <f>SUM(O4:O9)</f>
-        <v>0</v>
-      </c>
-      <c r="K14" t="s">
-        <v>71</v>
-      </c>
-      <c r="L14">
-        <v>46.232580877717901</v>
-      </c>
-      <c r="M14">
-        <v>46.243127016089062</v>
-      </c>
-      <c r="S14" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>186</v>
-      </c>
-      <c r="E15">
-        <f>SUM(P4:P9)</f>
-        <v>0</v>
-      </c>
-      <c r="K15" t="s">
-        <v>63</v>
-      </c>
-      <c r="L15">
-        <v>5.4435182877526831</v>
-      </c>
-      <c r="M15">
-        <v>5.5155923611825912</v>
-      </c>
-      <c r="S15" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>188</v>
-      </c>
-      <c r="E16">
-        <f>SUM(Q4:Q9)</f>
-        <v>8.0779356694631609E-27</v>
-      </c>
-      <c r="K16" t="s">
-        <v>67</v>
-      </c>
-      <c r="L16">
-        <v>3.0672134474127284</v>
-      </c>
-      <c r="M16">
-        <v>3.112817975691188</v>
-      </c>
-      <c r="S16" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K17" t="s">
-        <v>72</v>
-      </c>
-      <c r="L17">
-        <v>0.28956719904890593</v>
-      </c>
-      <c r="M17">
-        <v>0.28796770498141772</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>191</v>
-      </c>
-      <c r="B19" t="s">
-        <v>192</v>
-      </c>
-      <c r="C19" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>194</v>
-      </c>
-      <c r="B20">
-        <f>'FS No Vs 111'!BG31</f>
-        <v>7.2180533228467745</v>
-      </c>
-      <c r="C20">
-        <f>'FS No Vs 111'!AV30</f>
-        <v>55.456507868353405</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>195</v>
-      </c>
-      <c r="B21">
-        <f>'FS No Vp 111'!BC31</f>
-        <v>52.196130402976017</v>
-      </c>
-      <c r="C21">
-        <f>'FS No Vp 111'!AQ34</f>
-        <v>983.36124073377607</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>196</v>
-      </c>
-      <c r="B22">
-        <f>'FS No Vs 100'!BF31</f>
-        <v>15.798705890900674</v>
-      </c>
-      <c r="C22">
-        <f>'FS No Vs 100'!AQ32</f>
-        <v>18.827546785413528</v>
-      </c>
-      <c r="L22" t="s">
-        <v>202</v>
-      </c>
-      <c r="M22" t="s">
-        <v>201</v>
-      </c>
-      <c r="N22" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>197</v>
-      </c>
-      <c r="B23">
-        <f>'FS No Vp 100'!BH31</f>
-        <v>11.333238543153788</v>
-      </c>
-      <c r="C23">
-        <f>'FS No Vp 100'!AS32</f>
-        <v>74.737893177232252</v>
-      </c>
-      <c r="K23" t="s">
-        <v>62</v>
-      </c>
-      <c r="L23">
-        <v>239.89360432346049</v>
-      </c>
-      <c r="M23">
-        <v>239.510382116199</v>
-      </c>
-      <c r="N23">
-        <v>239.73960250702001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>198</v>
-      </c>
-      <c r="B24">
-        <f>SUM(B20:B23)</f>
-        <v>86.546128159877256</v>
-      </c>
-      <c r="C24">
-        <f>SUM(C20:C23)</f>
-        <v>1132.3831885647753</v>
-      </c>
-      <c r="K24" t="s">
-        <v>66</v>
-      </c>
-      <c r="L24">
-        <v>122.04281469011407</v>
-      </c>
-      <c r="M24">
-        <v>121.79137881717247</v>
-      </c>
-      <c r="N24">
-        <v>121.94076993310495</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>199</v>
-      </c>
-      <c r="B25">
-        <f>B24+C24</f>
-        <v>1218.9293167246526</v>
-      </c>
-      <c r="K25" t="s">
-        <v>71</v>
-      </c>
-      <c r="L25">
-        <v>46.221889892405528</v>
-      </c>
-      <c r="M25">
-        <v>46.243127016089062</v>
-      </c>
-      <c r="N25">
-        <v>46.232580870463721</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K26" t="s">
-        <v>63</v>
-      </c>
-      <c r="L26">
-        <v>5.3841194796800016</v>
-      </c>
-      <c r="M26">
-        <v>5.5155923611825912</v>
-      </c>
-      <c r="N26">
-        <v>5.4435182768766763</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K27" t="s">
-        <v>67</v>
-      </c>
-      <c r="L27">
-        <v>3.0296303147805537</v>
-      </c>
-      <c r="M27">
-        <v>3.112817975691188</v>
-      </c>
-      <c r="N27">
-        <v>3.0672134487654747</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K28" t="s">
-        <v>72</v>
-      </c>
-      <c r="L28">
-        <v>0.29107402544791877</v>
-      </c>
-      <c r="M28">
-        <v>0.28796770498141772</v>
-      </c>
-      <c r="N28">
-        <v>0.28956720143051184</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="M30" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M31" s="12">
-        <v>0.70399999999999996</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M32" s="12">
-        <v>0.70380627040878718</v>
-      </c>
-    </row>
-    <row r="33" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M33" s="12">
-        <v>0.70166388640963195</v>
-      </c>
-    </row>
-    <row r="34" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M34" s="12">
-        <v>0.70046889896090037</v>
-      </c>
-    </row>
-    <row r="35" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M35" s="24">
-        <v>0.69917394677785549</v>
-      </c>
-    </row>
-    <row r="36" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M36" s="12">
-        <v>0.69804545423270248</v>
-      </c>
-    </row>
-    <row r="37" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M37" s="12">
-        <v>0.6971320441092701</v>
-      </c>
-    </row>
-    <row r="38" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M38" s="12">
-        <v>0.69601338984367045</v>
-      </c>
-    </row>
-    <row r="39" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M39" s="12">
-        <v>0.69539727621518321</v>
-      </c>
-    </row>
-    <row r="40" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M40" s="12">
-        <v>0.69426566744215223</v>
-      </c>
-    </row>
-    <row r="41" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M41" s="12">
-        <v>0.69353731251708994</v>
-      </c>
-    </row>
-    <row r="42" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M42" s="12">
-        <v>0.69299062205044293</v>
-      </c>
-    </row>
-    <row r="43" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M43" s="12">
-        <v>0.69226271374904658</v>
-      </c>
-    </row>
-    <row r="44" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M44" s="12">
-        <v>0.69164775828557135</v>
-      </c>
-    </row>
-    <row r="45" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M45" s="36">
-        <v>0.69104384879900871</v>
-      </c>
-    </row>
-    <row r="46" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M46" s="12">
-        <v>0.690232937402526</v>
-      </c>
-    </row>
-    <row r="47" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M47" s="12">
-        <v>0.68988576586557904</v>
-      </c>
-    </row>
-    <row r="48" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M48" s="12">
-        <v>0.68964035968165227</v>
-      </c>
-    </row>
-    <row r="49" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M49" s="12">
-        <v>0.68920330986458733</v>
-      </c>
-    </row>
-    <row r="50" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M50" s="12">
-        <v>0.68862556359445315</v>
-      </c>
-    </row>
-    <row r="51" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M51" s="12">
-        <v>0.68833907152648766</v>
-      </c>
-    </row>
-    <row r="52" spans="13:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="M52" s="12">
-        <v>0.68814953473623941</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>